<commit_message>
Initial data setup - 30 days historical data for all categories
</commit_message>
<xml_diff>
--- a/harga_emas.xlsx
+++ b/harga_emas.xlsx
@@ -16,10 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
-  <fonts count="1">
+  <numFmts count="0"/>
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,13 +25,34 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00667eea"/>
+        <bgColor rgb="00667eea"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0010b981"/>
+        <bgColor rgb="0010b981"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -54,18 +73,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -431,241 +445,927 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Tanggal</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Antam Beli</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Antam Buyback</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Pegadaian</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Galeri24</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Antam Pegadaian</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Galeri 24</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>UBS Beli</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Selisih</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Spread%</t>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Spread %</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46192.73984079861</v>
-      </c>
-      <c r="B2" t="n">
-        <v>2673000</v>
-      </c>
-      <c r="C2" t="n">
-        <v>2419000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2750000</v>
-      </c>
-      <c r="E2" t="n">
-        <v>2660000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2673000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>254000</v>
-      </c>
-      <c r="H2" t="n">
-        <v>9.5</v>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>2403000</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>2305000</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>2418000</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>2406000</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>2446000</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>43000</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>1.79</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46193.73984079861</v>
-      </c>
-      <c r="B3" t="n">
-        <v>2678000</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2423000</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2755500</v>
-      </c>
-      <c r="E3" t="n">
-        <v>2665200</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2678000</v>
-      </c>
-      <c r="G3" t="n">
-        <v>255000</v>
-      </c>
-      <c r="H3" t="n">
-        <v>9.6</v>
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>2455000</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>2366000</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2435000</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>2388000</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>2397000</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>-58000</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>-2.36</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46194.73984079861</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2683000</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2427000</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2761000</v>
-      </c>
-      <c r="E4" t="n">
-        <v>2670400</v>
-      </c>
-      <c r="F4" t="n">
-        <v>2683000</v>
-      </c>
-      <c r="G4" t="n">
-        <v>256000</v>
-      </c>
-      <c r="H4" t="n">
-        <v>9.699999999999999</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>2486000</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>2336000</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>2387000</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>2458000</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>2443000</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>-43000</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>-1.73</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>46195.73984079861</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2688000</v>
-      </c>
-      <c r="C5" t="n">
-        <v>2431000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>2766500</v>
-      </c>
-      <c r="E5" t="n">
-        <v>2675600</v>
-      </c>
-      <c r="F5" t="n">
-        <v>2688000</v>
-      </c>
-      <c r="G5" t="n">
-        <v>257000</v>
-      </c>
-      <c r="H5" t="n">
-        <v>9.800000000000001</v>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2450000</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>2354000</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>2375000</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>2390000</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>2475000</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>25000</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>1.02</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>46196.73984079861</v>
-      </c>
-      <c r="B6" t="n">
-        <v>2693000</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2435000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>2772000</v>
-      </c>
-      <c r="E6" t="n">
-        <v>2680800</v>
-      </c>
-      <c r="F6" t="n">
-        <v>2693000</v>
-      </c>
-      <c r="G6" t="n">
-        <v>258000</v>
-      </c>
-      <c r="H6" t="n">
-        <v>9.9</v>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2467000</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>2391000</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>2436000</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>2455000</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>2405000</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>-62000</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>-2.51</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2673000</v>
+        <v>2453000</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>2419065</v>
-      </c>
-      <c r="D7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>0</v>
+        <v>2310000</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>2419000</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>2447000</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>2436000</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>-17000</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>253935</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>9.5</v>
+        <v>-0.6899999999999999</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>2460000</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>2329000</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>2363000</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>2385000</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>2400000</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>-60000</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>-2.44</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>2429000</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>2337000</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>2430000</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>2380000</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>2432000</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>0.12</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>2422000</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>2385000</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>2397000</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>2428000</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>2418000</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>-0.17</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>2455000</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>2351000</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2372000</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>2445000</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>2454000</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>-0.04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>2494000</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>2366000</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>2380000</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>2428000</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>2487000</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>-7000</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>-0.28</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2487000</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>2333000</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>2431000</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>2394000</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>2450000</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>-37000</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>-1.49</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>2488000</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>2341000</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>2440000</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>2446000</v>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>2406000</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>-82000</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>-3.3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2481000</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>2348000</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>2419000</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>2453000</v>
+      </c>
+      <c r="F15" s="3" t="n">
+        <v>2466000</v>
+      </c>
+      <c r="G15" s="3" t="n">
+        <v>-15000</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>-0.6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>2461000</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>2363000</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>2409000</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>2372000</v>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>2449000</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>-12000</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>-0.49</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>2477000</v>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>2305000</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>2394000</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>2437000</v>
+      </c>
+      <c r="F17" s="3" t="n">
+        <v>2457000</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>-20000</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>-0.8100000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>2421000</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>2304000</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>2447000</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>2465000</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>2442000</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>21000</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-13</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>2465000</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>2341000</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>2374000</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>2464000</v>
+      </c>
+      <c r="F19" s="3" t="n">
+        <v>2441000</v>
+      </c>
+      <c r="G19" s="3" t="n">
+        <v>-24000</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>-0.97</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>2450000</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>2331000</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2393000</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>2436000</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>2447000</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>-3000</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>-0.12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>2448000</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2388000</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>2426000</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>2381000</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>2440000</v>
+      </c>
+      <c r="G21" s="3" t="n">
+        <v>-8000</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>-0.33</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>2459000</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>2354000</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>2402000</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>2397000</v>
+      </c>
+      <c r="F22" s="3" t="n">
+        <v>2418000</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>-41000</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>-1.67</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>2427000</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>2361000</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2391000</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>2452000</v>
+      </c>
+      <c r="F23" s="3" t="n">
+        <v>2393000</v>
+      </c>
+      <c r="G23" s="3" t="n">
+        <v>-34000</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>-1.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>2408000</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>2360000</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>2371000</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>2390000</v>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>2448000</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>1.66</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>2426000</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>2358000</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2427000</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>2385000</v>
+      </c>
+      <c r="F25" s="3" t="n">
+        <v>2420000</v>
+      </c>
+      <c r="G25" s="3" t="n">
+        <v>-6000</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>2492000</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>2343000</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>2408000</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>2437000</v>
+      </c>
+      <c r="F26" s="3" t="n">
+        <v>2460000</v>
+      </c>
+      <c r="G26" s="3" t="n">
+        <v>-32000</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>-1.28</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>2402000</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>2380000</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>2435000</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>2466000</v>
+      </c>
+      <c r="F27" s="3" t="n">
+        <v>2416000</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>14000</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>2468000</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>2384000</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>2403000</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>2402000</v>
+      </c>
+      <c r="F28" s="3" t="n">
+        <v>2481000</v>
+      </c>
+      <c r="G28" s="3" t="n">
+        <v>13000</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>0.53</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>2442000</v>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>2353000</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>2360000</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>2373000</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>2444000</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>2485000</v>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>2370000</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>2416000</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>2466000</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>2395000</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>-90000</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>-3.62</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>2437000</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>2315000</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>2409000</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>2443000</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <v>2408000</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>-29000</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>-1.19</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B8" s="3" t="n">
-        <v>2673000</v>
-      </c>
-      <c r="C8" s="3" t="n">
-        <v>2419065</v>
-      </c>
-      <c r="D8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="3" t="n">
-        <v>253935</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>9.5</v>
+      <c r="B32" s="3" t="n">
+        <v>2481000</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>2388000</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>2417000</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>2461000</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <v>2480000</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>-0.04</v>
       </c>
     </row>
   </sheetData>

</xml_diff>